<commit_message>
Agrega logs de ejecución exitosa y con error
</commit_message>
<xml_diff>
--- a/salida/carga_novedades_20261026.xlsx
+++ b/salida/carga_novedades_20261026.xlsx
@@ -429,22 +429,22 @@
   <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="25" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="25" customWidth="1" min="8" max="8"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="19" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="16" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="21" customWidth="1" min="4" max="4"/>
+    <col width="29" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="29" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="22" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1167,14 +1167,14 @@
   <dimension ref="A1:H14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="17" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
     <col width="80" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="21" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1745,10 +1745,10 @@
   <dimension ref="A1:D3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="28" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="29" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1823,11 +1823,11 @@
   <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="33" customWidth="1" min="1" max="1"/>
-    <col width="71" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="21" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>